<commit_message>
Handbook Changes + CVS Change
</commit_message>
<xml_diff>
--- a/Assets/Resources/Excel sheets/Requests.xlsx
+++ b/Assets/Resources/Excel sheets/Requests.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29127"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\artem\Desktop\RMIT\RMIT sem 2 2026\GDS6\VANDERBILT\Assets\Resources\Excel sheets\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\GamesDesign2026\CAPSTONE\GITHUB\VANDERBILT\Assets\Resources\Excel sheets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8A8E6794-A571-4736-BF08-812A07D843D6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C928618A-D1BD-4BAD-92DC-CEE7A967F96F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="2055" windowWidth="30570" windowHeight="15270" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="34620" windowHeight="13900" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="246" uniqueCount="103">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="246" uniqueCount="102">
   <si>
     <t>Reward</t>
   </si>
@@ -73,9 +73,6 @@
   </si>
   <si>
     <t>Military</t>
-  </si>
-  <si>
-    <t>ResourceDepot</t>
   </si>
   <si>
     <t>LocationType</t>
@@ -705,23 +702,23 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:P60"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="3" width="23.42578125" customWidth="1"/>
-    <col min="4" max="4" width="21.140625" customWidth="1"/>
-    <col min="5" max="5" width="8.85546875" customWidth="1"/>
-    <col min="6" max="6" width="15.42578125" customWidth="1"/>
-    <col min="7" max="7" width="10.42578125" customWidth="1"/>
+    <col min="1" max="3" width="23.453125" customWidth="1"/>
+    <col min="4" max="4" width="21.1796875" customWidth="1"/>
+    <col min="5" max="5" width="8.81640625" customWidth="1"/>
+    <col min="6" max="6" width="15.453125" customWidth="1"/>
+    <col min="7" max="7" width="10.453125" customWidth="1"/>
     <col min="8" max="8" width="15" customWidth="1"/>
-    <col min="9" max="9" width="23.5703125" customWidth="1"/>
-    <col min="10" max="10" width="12.7109375" customWidth="1"/>
-    <col min="11" max="11" width="11.85546875" customWidth="1"/>
-    <col min="12" max="12" width="14.140625" customWidth="1"/>
-    <col min="13" max="13" width="15.140625" customWidth="1"/>
-    <col min="14" max="14" width="15.42578125" customWidth="1"/>
+    <col min="9" max="9" width="23.54296875" customWidth="1"/>
+    <col min="10" max="10" width="12.7265625" customWidth="1"/>
+    <col min="11" max="11" width="11.81640625" customWidth="1"/>
+    <col min="12" max="12" width="14.1796875" customWidth="1"/>
+    <col min="13" max="13" width="15.1796875" customWidth="1"/>
+    <col min="14" max="14" width="15.453125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" ht="20.25" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:16" ht="20.25" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">
         <v>5</v>
       </c>
@@ -759,27 +756,27 @@
         <v>10</v>
       </c>
       <c r="M1" s="1" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="N1" s="1" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:16" ht="60" customHeight="1" thickTop="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:16" ht="60" customHeight="1" thickTop="1" x14ac:dyDescent="0.35">
       <c r="A2" s="3" t="s">
         <v>13</v>
       </c>
       <c r="B2" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="C2" s="3" t="s">
         <v>18</v>
-      </c>
-      <c r="C2" s="3" t="s">
-        <v>19</v>
       </c>
       <c r="D2" s="3">
         <v>40</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F2" s="3">
         <v>80</v>
@@ -788,10 +785,10 @@
         <v>8</v>
       </c>
       <c r="H2" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="I2" s="3" t="s">
         <v>21</v>
-      </c>
-      <c r="I2" s="3" t="s">
-        <v>22</v>
       </c>
       <c r="J2" s="3">
         <v>5</v>
@@ -803,27 +800,27 @@
         <v>1</v>
       </c>
       <c r="M2" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="N2" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="N2" s="3" t="s">
+    </row>
+    <row r="3" spans="1:16" ht="60" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A3" s="3" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="3" spans="1:16" ht="60" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="3" t="s">
+      <c r="B3" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="C3" s="3" t="s">
         <v>25</v>
-      </c>
-      <c r="B3" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="C3" s="3" t="s">
-        <v>26</v>
       </c>
       <c r="D3" s="3">
         <v>20</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F3" s="3">
         <v>100</v>
@@ -832,10 +829,10 @@
         <v>6</v>
       </c>
       <c r="H3" s="3" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="I3" s="3" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="J3" s="3">
         <v>8</v>
@@ -850,24 +847,24 @@
         <v>14</v>
       </c>
       <c r="N3" s="3" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="4" spans="1:16" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="4" spans="1:16" ht="60" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A4" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="C4" s="3" t="s">
         <v>28</v>
-      </c>
-      <c r="B4" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="C4" s="3" t="s">
-        <v>29</v>
       </c>
       <c r="D4" s="3">
         <v>15</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F4" s="3">
         <v>120</v>
@@ -876,10 +873,10 @@
         <v>10</v>
       </c>
       <c r="H4" s="3" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="I4" s="3" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="J4" s="3">
         <v>10</v>
@@ -891,27 +888,27 @@
         <v>0</v>
       </c>
       <c r="M4" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="N4" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="N4" s="3" t="s">
+    </row>
+    <row r="5" spans="1:16" ht="60" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A5" s="3" t="s">
         <v>32</v>
       </c>
-    </row>
-    <row r="5" spans="1:16" ht="60" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="3" t="s">
+      <c r="B5" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="C5" s="3" t="s">
         <v>33</v>
-      </c>
-      <c r="B5" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="C5" s="3" t="s">
-        <v>34</v>
       </c>
       <c r="D5" s="3">
         <v>30</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F5" s="3">
         <v>90</v>
@@ -920,10 +917,10 @@
         <v>7</v>
       </c>
       <c r="H5" s="3" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="I5" s="3" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="J5" s="3">
         <v>7</v>
@@ -935,27 +932,27 @@
         <v>1</v>
       </c>
       <c r="M5" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="N5" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="N5" s="3" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="6" spans="1:16" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="6" spans="1:16" ht="60" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A6" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="B6" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="C6" s="3" t="s">
         <v>36</v>
-      </c>
-      <c r="B6" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="C6" s="3" t="s">
-        <v>37</v>
       </c>
       <c r="D6" s="3">
         <v>10</v>
       </c>
       <c r="E6" s="3" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F6" s="3">
         <v>150</v>
@@ -964,10 +961,10 @@
         <v>9</v>
       </c>
       <c r="H6" s="3" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="I6" s="3" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="J6" s="3">
         <v>12</v>
@@ -982,24 +979,24 @@
         <v>15</v>
       </c>
       <c r="N6" s="3" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="7" spans="1:16" ht="60" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A7" s="3" t="s">
         <v>39</v>
       </c>
-    </row>
-    <row r="7" spans="1:16" ht="60" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="3" t="s">
-        <v>40</v>
-      </c>
       <c r="B7" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="C7" s="3" t="s">
         <v>18</v>
-      </c>
-      <c r="C7" s="3" t="s">
-        <v>19</v>
       </c>
       <c r="D7" s="3">
         <v>60</v>
       </c>
       <c r="E7" s="3" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="F7" s="3">
         <v>10</v>
@@ -1008,10 +1005,10 @@
         <v>12</v>
       </c>
       <c r="H7" s="3" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="I7" s="3" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="J7" s="3">
         <v>8</v>
@@ -1023,29 +1020,29 @@
         <v>1</v>
       </c>
       <c r="M7" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="N7" s="3" t="s">
         <v>23</v>
-      </c>
-      <c r="N7" s="3" t="s">
-        <v>24</v>
       </c>
       <c r="O7" s="2"/>
       <c r="P7" s="2"/>
     </row>
-    <row r="8" spans="1:16" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:16" ht="60" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A8" s="3" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="D8" s="3">
         <v>20</v>
       </c>
       <c r="E8" s="3" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F8" s="3">
         <v>110</v>
@@ -1054,10 +1051,10 @@
         <v>6</v>
       </c>
       <c r="H8" s="3" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="I8" s="3" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="J8" s="3">
         <v>10</v>
@@ -1072,26 +1069,26 @@
         <v>14</v>
       </c>
       <c r="N8" s="3" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="O8" s="3"/>
       <c r="P8" s="3"/>
     </row>
-    <row r="9" spans="1:16" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:16" ht="60" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A9" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="B9" s="3" t="s">
         <v>45</v>
       </c>
-      <c r="B9" s="3" t="s">
-        <v>46</v>
-      </c>
       <c r="C9" s="3" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="D9" s="3">
         <v>25</v>
       </c>
       <c r="E9" s="3" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F9" s="3">
         <v>200</v>
@@ -1100,10 +1097,10 @@
         <v>10</v>
       </c>
       <c r="H9" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="I9" s="3" t="s">
         <v>47</v>
-      </c>
-      <c r="I9" s="3" t="s">
-        <v>48</v>
       </c>
       <c r="J9" s="3">
         <v>6</v>
@@ -1115,29 +1112,29 @@
         <v>1</v>
       </c>
       <c r="M9" s="3" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="N9" s="3" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="O9" s="3"/>
       <c r="P9" s="3"/>
     </row>
-    <row r="10" spans="1:16" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:16" ht="60" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A10" s="3" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="D10" s="3">
         <v>50</v>
       </c>
       <c r="E10" s="3" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F10" s="3">
         <v>180</v>
@@ -1146,10 +1143,10 @@
         <v>8</v>
       </c>
       <c r="H10" s="3" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="I10" s="3" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="J10" s="3">
         <v>5</v>
@@ -1161,29 +1158,29 @@
         <v>1</v>
       </c>
       <c r="M10" s="3" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="N10" s="3" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="O10" s="3"/>
       <c r="P10" s="3"/>
     </row>
-    <row r="11" spans="1:16" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:16" ht="60" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A11" s="3" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="D11" s="3">
         <v>35</v>
       </c>
       <c r="E11" s="3" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F11" s="3">
         <v>160</v>
@@ -1192,10 +1189,10 @@
         <v>7</v>
       </c>
       <c r="H11" s="3" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="I11" s="3" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="J11" s="3">
         <v>4</v>
@@ -1207,29 +1204,29 @@
         <v>1</v>
       </c>
       <c r="M11" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="N11" s="3" t="s">
         <v>23</v>
-      </c>
-      <c r="N11" s="3" t="s">
-        <v>24</v>
       </c>
       <c r="O11" s="3"/>
       <c r="P11" s="3"/>
     </row>
-    <row r="12" spans="1:16" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:16" ht="60" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A12" s="3" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C12" s="3" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="D12" s="3">
         <v>15</v>
       </c>
       <c r="E12" s="3" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F12" s="3">
         <v>220</v>
@@ -1238,10 +1235,10 @@
         <v>5</v>
       </c>
       <c r="H12" s="3" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="I12" s="3" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="J12" s="3">
         <v>8</v>
@@ -1256,26 +1253,26 @@
         <v>14</v>
       </c>
       <c r="N12" s="3" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="O12" s="3"/>
       <c r="P12" s="3"/>
     </row>
-    <row r="13" spans="1:16" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:16" ht="60" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A13" s="3" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C13" s="3" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D13" s="3">
         <v>20</v>
       </c>
       <c r="E13" s="3" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F13" s="3">
         <v>250</v>
@@ -1284,10 +1281,10 @@
         <v>9</v>
       </c>
       <c r="H13" s="3" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="I13" s="3" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="J13" s="3">
         <v>15</v>
@@ -1302,26 +1299,26 @@
         <v>15</v>
       </c>
       <c r="N13" s="3" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="O13" s="3"/>
       <c r="P13" s="3"/>
     </row>
-    <row r="14" spans="1:16" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:16" ht="60" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A14" s="3" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C14" s="3" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="D14" s="3">
         <v>30</v>
       </c>
       <c r="E14" s="3" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="F14" s="3">
         <v>25</v>
@@ -1330,10 +1327,10 @@
         <v>12</v>
       </c>
       <c r="H14" s="3" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="I14" s="3" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="J14" s="3">
         <v>7</v>
@@ -1345,29 +1342,29 @@
         <v>1</v>
       </c>
       <c r="M14" s="3" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="N14" s="3" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="O14" s="3"/>
       <c r="P14" s="3"/>
     </row>
-    <row r="15" spans="1:16" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:16" ht="60" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A15" s="3" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C15" s="3" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="D15" s="3">
         <v>45</v>
       </c>
       <c r="E15" s="3" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F15" s="3">
         <v>140</v>
@@ -1376,10 +1373,10 @@
         <v>6</v>
       </c>
       <c r="H15" s="3" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="I15" s="3" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="J15" s="3">
         <v>6</v>
@@ -1391,29 +1388,29 @@
         <v>1</v>
       </c>
       <c r="M15" s="3" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="N15" s="3" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="O15" s="3"/>
       <c r="P15" s="3"/>
     </row>
-    <row r="16" spans="1:16" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:16" ht="60" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A16" s="3" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C16" s="3" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="D16" s="3">
         <v>10</v>
       </c>
       <c r="E16" s="3" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="F16" s="3">
         <v>15</v>
@@ -1422,10 +1419,10 @@
         <v>5</v>
       </c>
       <c r="H16" s="3" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="I16" s="3" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="J16" s="3">
         <v>5</v>
@@ -1437,29 +1434,29 @@
         <v>1</v>
       </c>
       <c r="M16" s="3" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="N16" s="3" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="O16" s="3"/>
       <c r="P16" s="3"/>
     </row>
-    <row r="17" spans="1:16" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:16" ht="60" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A17" s="3" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C17" s="3" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D17" s="3">
         <v>15</v>
       </c>
       <c r="E17" s="3" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F17" s="3">
         <v>180</v>
@@ -1468,10 +1465,10 @@
         <v>8</v>
       </c>
       <c r="H17" s="3" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="I17" s="3" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="J17" s="3">
         <v>10</v>
@@ -1486,26 +1483,26 @@
         <v>15</v>
       </c>
       <c r="N17" s="3" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="O17" s="3"/>
       <c r="P17" s="3"/>
     </row>
-    <row r="18" spans="1:16" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:16" ht="60" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A18" s="3" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="B18" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="C18" s="3" t="s">
         <v>18</v>
-      </c>
-      <c r="C18" s="3" t="s">
-        <v>19</v>
       </c>
       <c r="D18" s="3">
         <v>50</v>
       </c>
       <c r="E18" s="3" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F18" s="3">
         <v>130</v>
@@ -1514,10 +1511,10 @@
         <v>10</v>
       </c>
       <c r="H18" s="3" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="I18" s="3" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="J18" s="3">
         <v>12</v>
@@ -1529,29 +1526,29 @@
         <v>0</v>
       </c>
       <c r="M18" s="3" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="N18" s="3" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="O18" s="3"/>
       <c r="P18" s="3"/>
     </row>
-    <row r="19" spans="1:16" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:16" ht="60" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A19" s="3" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B19" s="3" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C19" s="3" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="D19" s="3">
         <v>30</v>
       </c>
       <c r="E19" s="3" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F19" s="3">
         <v>180</v>
@@ -1560,10 +1557,10 @@
         <v>7</v>
       </c>
       <c r="H19" s="3" t="s">
+        <v>71</v>
+      </c>
+      <c r="I19" s="3" t="s">
         <v>72</v>
-      </c>
-      <c r="I19" s="3" t="s">
-        <v>73</v>
       </c>
       <c r="J19" s="3">
         <v>10</v>
@@ -1578,26 +1575,26 @@
         <v>14</v>
       </c>
       <c r="N19" s="3" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="O19" s="3"/>
       <c r="P19" s="3"/>
     </row>
-    <row r="20" spans="1:16" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:16" ht="60" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A20" s="3" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="B20" s="3" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C20" s="3" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="D20" s="3">
         <v>20</v>
       </c>
       <c r="E20" s="3" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="F20" s="3">
         <v>30</v>
@@ -1606,10 +1603,10 @@
         <v>9</v>
       </c>
       <c r="H20" s="3" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="I20" s="3" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="J20" s="3">
         <v>9</v>
@@ -1621,29 +1618,29 @@
         <v>1</v>
       </c>
       <c r="M20" s="3" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="N20" s="3" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="O20" s="3"/>
       <c r="P20" s="3"/>
     </row>
-    <row r="21" spans="1:16" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:16" ht="60" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A21" s="3" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="B21" s="3" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C21" s="3" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="D21" s="3">
         <v>40</v>
       </c>
       <c r="E21" s="3" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F21" s="3">
         <v>160</v>
@@ -1652,10 +1649,10 @@
         <v>8</v>
       </c>
       <c r="H21" s="3" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="I21" s="3" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="J21" s="3">
         <v>12</v>
@@ -1667,29 +1664,29 @@
         <v>0</v>
       </c>
       <c r="M21" s="3" t="s">
-        <v>16</v>
+        <v>22</v>
       </c>
       <c r="N21" s="3" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="O21" s="3"/>
       <c r="P21" s="3"/>
     </row>
-    <row r="22" spans="1:16" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:16" ht="60" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A22" s="3" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B22" s="3" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C22" s="3" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D22" s="3">
         <v>8</v>
       </c>
       <c r="E22" s="3" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F22" s="3">
         <v>200</v>
@@ -1698,10 +1695,10 @@
         <v>6</v>
       </c>
       <c r="H22" s="3" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="I22" s="3" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="J22" s="3">
         <v>15</v>
@@ -1716,26 +1713,26 @@
         <v>15</v>
       </c>
       <c r="N22" s="3" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="O22" s="3"/>
       <c r="P22" s="3"/>
     </row>
-    <row r="23" spans="1:16" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:16" ht="60" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A23" s="3" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="B23" s="3" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C23" s="3" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="D23" s="3">
         <v>70</v>
       </c>
       <c r="E23" s="3" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F23" s="3">
         <v>300</v>
@@ -1744,10 +1741,10 @@
         <v>12</v>
       </c>
       <c r="H23" s="3" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="I23" s="3" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="J23" s="3">
         <v>8</v>
@@ -1759,29 +1756,29 @@
         <v>1</v>
       </c>
       <c r="M23" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="N23" s="3" t="s">
         <v>23</v>
-      </c>
-      <c r="N23" s="3" t="s">
-        <v>24</v>
       </c>
       <c r="O23" s="3"/>
       <c r="P23" s="3"/>
     </row>
-    <row r="24" spans="1:16" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:16" ht="60" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A24" s="3" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="B24" s="3" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C24" s="3" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="D24" s="3">
         <v>25</v>
       </c>
       <c r="E24" s="3" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F24" s="3">
         <v>280</v>
@@ -1790,10 +1787,10 @@
         <v>6</v>
       </c>
       <c r="H24" s="3" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="I24" s="3" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="J24" s="3">
         <v>7</v>
@@ -1808,26 +1805,26 @@
         <v>14</v>
       </c>
       <c r="N24" s="3" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="O24" s="3"/>
       <c r="P24" s="3"/>
     </row>
-    <row r="25" spans="1:16" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:16" ht="60" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A25" s="3" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="B25" s="3" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C25" s="3" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="D25" s="3">
         <v>40</v>
       </c>
       <c r="E25" s="3" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F25" s="3">
         <v>350</v>
@@ -1836,10 +1833,10 @@
         <v>12</v>
       </c>
       <c r="H25" s="3" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="I25" s="3" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="J25" s="3">
         <v>12</v>
@@ -1851,29 +1848,29 @@
         <v>0</v>
       </c>
       <c r="M25" s="3" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="N25" s="3" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="O25" s="3"/>
       <c r="P25" s="3"/>
     </row>
-    <row r="26" spans="1:16" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:16" ht="60" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A26" s="3" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="B26" s="3" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C26" s="3" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="D26" s="3">
         <v>60</v>
       </c>
       <c r="E26" s="3" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F26" s="3">
         <v>300</v>
@@ -1882,10 +1879,10 @@
         <v>10</v>
       </c>
       <c r="H26" s="3" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="I26" s="3" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="J26" s="3">
         <v>10</v>
@@ -1897,29 +1894,29 @@
         <v>1</v>
       </c>
       <c r="M26" s="3" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="N26" s="3" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="O26" s="3"/>
       <c r="P26" s="3"/>
     </row>
-    <row r="27" spans="1:16" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:16" ht="60" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A27" s="3" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="B27" s="3" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C27" s="3" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D27" s="3">
         <v>30</v>
       </c>
       <c r="E27" s="3" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F27" s="3">
         <v>400</v>
@@ -1928,10 +1925,10 @@
         <v>9</v>
       </c>
       <c r="H27" s="3" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="I27" s="3" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="J27" s="3">
         <v>20</v>
@@ -1946,26 +1943,26 @@
         <v>15</v>
       </c>
       <c r="N27" s="3" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="O27" s="3"/>
       <c r="P27" s="3"/>
     </row>
-    <row r="28" spans="1:16" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:16" ht="60" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A28" s="3" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="B28" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="C28" s="3" t="s">
         <v>18</v>
-      </c>
-      <c r="C28" s="3" t="s">
-        <v>19</v>
       </c>
       <c r="D28" s="3">
         <v>30</v>
       </c>
       <c r="E28" s="3" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="F28" s="3">
         <v>15</v>
@@ -1974,10 +1971,10 @@
         <v>10</v>
       </c>
       <c r="H28" s="3" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="I28" s="3" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="J28" s="3">
         <v>6</v>
@@ -1989,29 +1986,29 @@
         <v>1</v>
       </c>
       <c r="M28" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="N28" s="3" t="s">
         <v>23</v>
-      </c>
-      <c r="N28" s="3" t="s">
-        <v>24</v>
       </c>
       <c r="O28" s="3"/>
       <c r="P28" s="3"/>
     </row>
-    <row r="29" spans="1:16" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:16" ht="60" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A29" s="3" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="B29" s="3" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C29" s="3" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="D29" s="3">
         <v>12</v>
       </c>
       <c r="E29" s="3" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="F29" s="3">
         <v>20</v>
@@ -2020,10 +2017,10 @@
         <v>7</v>
       </c>
       <c r="H29" s="3" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="I29" s="3" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="J29" s="3">
         <v>7</v>
@@ -2035,29 +2032,29 @@
         <v>1</v>
       </c>
       <c r="M29" s="3" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="N29" s="3" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="O29" s="3"/>
       <c r="P29" s="3"/>
     </row>
-    <row r="30" spans="1:16" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:16" ht="60" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A30" s="3" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="B30" s="3" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C30" s="3" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D30" s="3">
         <v>12</v>
       </c>
       <c r="E30" s="3" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="F30" s="3">
         <v>40</v>
@@ -2066,10 +2063,10 @@
         <v>8</v>
       </c>
       <c r="H30" s="3" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="I30" s="3" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="J30" s="3">
         <v>18</v>
@@ -2084,47 +2081,47 @@
         <v>15</v>
       </c>
       <c r="N30" s="3" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="O30" s="3"/>
       <c r="P30" s="3"/>
     </row>
-    <row r="31" spans="1:16" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:16" ht="60" customHeight="1" x14ac:dyDescent="0.35">
       <c r="O31" s="3"/>
       <c r="P31" s="3"/>
     </row>
-    <row r="32" spans="1:16" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:16" ht="60" customHeight="1" x14ac:dyDescent="0.35">
       <c r="O32" s="3"/>
       <c r="P32" s="3"/>
     </row>
-    <row r="33" ht="60" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="34" ht="60" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="35" ht="60" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="36" ht="60" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="37" ht="60" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="38" ht="60" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="39" ht="60" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="40" ht="60" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="41" ht="60" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="42" ht="60" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="43" ht="60" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="44" ht="60" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="45" ht="60" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="46" ht="60" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="47" ht="60" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="48" ht="60" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="49" ht="60" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="50" ht="60" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="51" ht="60" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="52" ht="60" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="53" ht="60" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="54" ht="60" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="55" ht="60" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="56" ht="60" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="57" ht="60" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="58" ht="60" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="59" ht="60" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="60" ht="60" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="33" ht="60" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="34" ht="60" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="35" ht="60" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="36" ht="60" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="37" ht="60" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="38" ht="60" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="39" ht="60" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="40" ht="60" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="41" ht="60" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="42" ht="60" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="43" ht="60" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="44" ht="60" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="45" ht="60" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="46" ht="60" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="47" ht="60" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="48" ht="60" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="49" ht="60" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="50" ht="60" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="51" ht="60" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="52" ht="60" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="53" ht="60" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="54" ht="60" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="55" ht="60" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="56" ht="60" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="57" ht="60" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="58" ht="60" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="59" ht="60" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="60" ht="60" customHeight="1" x14ac:dyDescent="0.35"/>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>